<commit_message>
Resolved Cost Calculator Failed Test cases - 14-04-2026
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/16_Cost_Calculator/CostCalculator/01_CostCalculatorTest.xlsx
+++ b/src/test/resources/testdata/Modules/16_Cost_Calculator/CostCalculator/01_CostCalculatorTest.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\16_Cost_Calculator\CostCalculator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\16_Cost_Calculator\CostCalculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC881919-D060-41F8-8C45-01CF72D7E67A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CACB115-C7FE-4736-9F49-D0860094E66B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="2" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
   <sheets>
     <sheet name="TestCases" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="237">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -62,54 +62,6 @@
   </si>
   <si>
     <t>2602000005</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_01</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_02</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_03</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_04</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_05</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_06</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_07</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_08</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_09</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_10</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_11</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_12</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_13</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_14</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_15</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_16</t>
   </si>
   <si>
     <t>Customer_name</t>
@@ -288,12 +240,6 @@
 verify_ui_title</t>
   </si>
   <si>
-    <t>CostCalculatorTest_17</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_18</t>
-  </si>
-  <si>
     <t>Delete and Add material</t>
   </si>
   <si>
@@ -415,10 +361,6 @@
   </si>
   <si>
     <t>Electical</t>
-  </si>
-  <si>
-    <t>click_on_next
-click_on_dream_gift</t>
   </si>
   <si>
     <t>Verify costings</t>
@@ -444,68 +386,383 @@
 click_on_next</t>
   </si>
   <si>
-    <t>CostCalculatorTest_19</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_20</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_21</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_22</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_23</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_24</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_25</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_26</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_27</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_28</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_30</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_31</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_32</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_33</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_34</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_35</t>
-  </si>
-  <si>
-    <t>CostCalculatorTest_37</t>
-  </si>
-  <si>
-    <t>click_on_next
-click_on_next
-verify_ui_title</t>
-  </si>
-  <si>
-    <t>click_on_next
-click_on_next</t>
-  </si>
-  <si>
     <t>click_on_delete
 click_on_add</t>
+  </si>
+  <si>
+    <t>click_cost_calculator
+fill_details_to_add_project_details_all
+add_project_quantities
+click_on_next</t>
+  </si>
+  <si>
+    <t>click_cost_calculator
+fill_details_to_add_project_details_all
+add_project_quantities_test_2
+click_on_next</t>
+  </si>
+  <si>
+    <t>Plywoods</t>
+  </si>
+  <si>
+    <t>click_on_next
+verify_materials_water_tank</t>
+  </si>
+  <si>
+    <t>verify_materials_cables</t>
+  </si>
+  <si>
+    <t>verify_materials_electrical_fittings</t>
+  </si>
+  <si>
+    <t>verify_materials_water_tank</t>
+  </si>
+  <si>
+    <t>verify_materials_tmt</t>
+  </si>
+  <si>
+    <t>verify_materials_cement</t>
+  </si>
+  <si>
+    <t>verify_materials_construction_chemicals</t>
+  </si>
+  <si>
+    <t>verify_materials_interior_paint</t>
+  </si>
+  <si>
+    <t>verify_materials_exterior_paint</t>
+  </si>
+  <si>
+    <t>verify_materials_primer</t>
+  </si>
+  <si>
+    <t>verify_materials_putty</t>
+  </si>
+  <si>
+    <t>verify_materials_doors</t>
+  </si>
+  <si>
+    <t>verify_materials_locks</t>
+  </si>
+  <si>
+    <t>verify_materials_windows</t>
+  </si>
+  <si>
+    <t>verify_materials_plywoods</t>
+  </si>
+  <si>
+    <t>verify_materials_laminates</t>
+  </si>
+  <si>
+    <t>verify_materials_pipes</t>
+  </si>
+  <si>
+    <t>verify_materials_tiles</t>
+  </si>
+  <si>
+    <t>verify_materials_sanitary_ware</t>
+  </si>
+  <si>
+    <t>verify_materials_bathroom_fittings</t>
+  </si>
+  <si>
+    <t>click_on_next
+verify_costing_plumbing</t>
+  </si>
+  <si>
+    <t>verify_costing_civil_work</t>
+  </si>
+  <si>
+    <t>verify_costing_paint_work</t>
+  </si>
+  <si>
+    <t>verify_costing_carpentary</t>
+  </si>
+  <si>
+    <t>verify_costing_electrical</t>
+  </si>
+  <si>
+    <t>verify_costing_dream_gift_electrical</t>
+  </si>
+  <si>
+    <t>verify_costing_dream_gift_carpentary</t>
+  </si>
+  <si>
+    <t>verify_costing_dream_gift_paint_work</t>
+  </si>
+  <si>
+    <t>verify_costing_dream_gift_civil_work</t>
+  </si>
+  <si>
+    <t>verify_costing_dream_gift_plumbing</t>
+  </si>
+  <si>
+    <t>click_on_next
+verify_ui_title</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_01</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_02</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_03</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_04</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_05</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_06</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_07</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_08</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_09</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_10</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_11</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_12</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_13</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_14</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_15</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_16</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_17</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_18</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest01_19</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_01</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_02</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_03</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_04</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_05</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_06</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_07</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_08</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_09</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_10</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_11</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_12</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_13</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_14</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_15</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_16</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_17</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_18</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_19</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_20</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_21</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_22</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_23</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_24</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_25</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_26</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_27</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_28</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_29</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_30</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_31</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_32</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_33</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_34</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest02_35</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_01</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_02</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_03</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_04</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_05</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_06</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_07</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_08</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_09</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_10</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_11</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_12</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_13</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_14</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_15</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_16</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_17</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_18</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_19</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_20</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_21</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_22</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_23</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_24</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_25</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_26</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_27</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_28</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_29</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_30</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_31</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_32</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_33</t>
+  </si>
+  <si>
+    <t>CostCalculatorTest03_34</t>
   </si>
   <si>
     <t>click_on_dream_gift
@@ -515,111 +772,9 @@
 click_exit_ok</t>
   </si>
   <si>
-    <t>click_cost_calculator
-fill_details_to_add_project_details_all
-add_project_quantities
-click_on_next</t>
-  </si>
-  <si>
-    <t>click_cost_calculator
-fill_details_to_add_project_details_all
-add_project_quantities_test_2
-click_on_next</t>
-  </si>
-  <si>
-    <t>Plywoods</t>
-  </si>
-  <si>
     <t>click_on_next
-verify_materials_water_tank</t>
-  </si>
-  <si>
-    <t>verify_materials_cables</t>
-  </si>
-  <si>
-    <t>verify_materials_electrical_fittings</t>
-  </si>
-  <si>
-    <t>verify_materials_water_tank</t>
-  </si>
-  <si>
-    <t>verify_materials_tmt</t>
-  </si>
-  <si>
-    <t>verify_materials_cement</t>
-  </si>
-  <si>
-    <t>verify_materials_construction_chemicals</t>
-  </si>
-  <si>
-    <t>verify_materials_interior_paint</t>
-  </si>
-  <si>
-    <t>verify_materials_exterior_paint</t>
-  </si>
-  <si>
-    <t>verify_materials_primer</t>
-  </si>
-  <si>
-    <t>verify_materials_putty</t>
-  </si>
-  <si>
-    <t>verify_materials_doors</t>
-  </si>
-  <si>
-    <t>verify_materials_locks</t>
-  </si>
-  <si>
-    <t>verify_materials_windows</t>
-  </si>
-  <si>
-    <t>verify_materials_plywoods</t>
-  </si>
-  <si>
-    <t>verify_materials_laminates</t>
-  </si>
-  <si>
-    <t>verify_materials_pipes</t>
-  </si>
-  <si>
-    <t>verify_materials_tiles</t>
-  </si>
-  <si>
-    <t>verify_materials_sanitary_ware</t>
-  </si>
-  <si>
-    <t>verify_materials_bathroom_fittings</t>
-  </si>
-  <si>
-    <t>click_on_next
-verify_costing_plumbing</t>
-  </si>
-  <si>
-    <t>verify_costing_civil_work</t>
-  </si>
-  <si>
-    <t>verify_costing_paint_work</t>
-  </si>
-  <si>
-    <t>verify_costing_carpentary</t>
-  </si>
-  <si>
-    <t>verify_costing_electrical</t>
-  </si>
-  <si>
-    <t>verify_costing_dream_gift_electrical</t>
-  </si>
-  <si>
-    <t>verify_costing_dream_gift_carpentary</t>
-  </si>
-  <si>
-    <t>verify_costing_dream_gift_paint_work</t>
-  </si>
-  <si>
-    <t>verify_costing_dream_gift_civil_work</t>
-  </si>
-  <si>
-    <t>verify_costing_dream_gift_plumbing</t>
+click_on_dream_gift
+click_on_dream_gift</t>
   </si>
 </sst>
 </file>
@@ -627,7 +782,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="6" formatCode="&quot;₹&quot;\ #,##0;[Red]&quot;₹&quot;\ \-#,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0;[Red]&quot;₹&quot;\ \-#,##0"/>
   </numFmts>
   <fonts count="24" x14ac:knownFonts="1">
     <font>
@@ -1288,7 +1443,7 @@
     <xf numFmtId="49" fontId="18" fillId="0" borderId="15" xfId="42" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1711,25 +1866,25 @@
         <v>3</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="J1" s="12" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="M1" s="11" t="s">
         <v>2</v>
@@ -1743,16 +1898,16 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>147</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="F2" s="14"/>
       <c r="G2" s="15"/>
@@ -1771,16 +1926,16 @@
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>148</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="1"/>
@@ -1790,7 +1945,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>5</v>
@@ -1801,32 +1956,32 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>149</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="H4" s="19" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
       <c r="M4" s="1" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>5</v>
@@ -1837,32 +1992,32 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>150</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="G5" s="19" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="H5" s="19" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="I5" s="19"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
       <c r="M5" s="1" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="N5" s="1" t="s">
         <v>5</v>
@@ -1873,34 +2028,34 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>151</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="G6" s="19" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="H6" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="19" t="s">
         <v>54</v>
-      </c>
-      <c r="I6" s="19" t="s">
-        <v>70</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="1" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="N6" s="1" t="s">
         <v>5</v>
@@ -1911,16 +2066,16 @@
         <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>14</v>
+        <v>152</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="F7" s="10"/>
       <c r="G7" s="1"/>
@@ -1930,10 +2085,10 @@
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
       <c r="M7" s="1" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>75</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="29" x14ac:dyDescent="0.35">
@@ -1941,16 +2096,16 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>15</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>31</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -1969,16 +2124,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E9" s="8" t="s">
         <v>16</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="8" t="s">
-        <v>32</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
@@ -1988,27 +2143,27 @@
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
       <c r="M9" s="1" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="N9" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>17</v>
+        <v>155</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F10" s="9"/>
       <c r="G10" s="1"/>
@@ -2018,7 +2173,7 @@
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
       <c r="M10" s="1" t="s">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="N10" s="1" t="s">
         <v>5</v>
@@ -2029,16 +2184,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
+        <v>156</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>150</v>
+        <v>112</v>
       </c>
       <c r="F11" s="9"/>
       <c r="G11" s="1"/>
@@ -2048,7 +2203,7 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="N11" s="1" t="s">
         <v>5</v>
@@ -2059,29 +2214,29 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>157</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
       <c r="M12" s="1"/>
       <c r="N12" s="1" t="s">
@@ -2093,16 +2248,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>20</v>
+        <v>158</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
@@ -2111,28 +2266,28 @@
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="M13" s="1"/>
       <c r="N13" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>21</v>
+        <v>159</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>149</v>
+        <v>18</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -2151,16 +2306,16 @@
         <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -2170,7 +2325,7 @@
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="1" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="N15" s="1" t="s">
         <v>5</v>
@@ -2181,16 +2336,16 @@
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>23</v>
+        <v>161</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="F16" s="10"/>
       <c r="G16" s="1"/>
@@ -2209,16 +2364,16 @@
         <v>8</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>24</v>
+        <v>162</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="F17" s="10"/>
       <c r="G17" s="1"/>
@@ -2228,7 +2383,7 @@
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="N17" s="1" t="s">
         <v>5</v>
@@ -2239,16 +2394,16 @@
         <v>8</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>80</v>
+        <v>163</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>151</v>
+        <v>235</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="1"/>
@@ -2267,16 +2422,16 @@
         <v>8</v>
       </c>
       <c r="B19" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>63</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E19" s="8" t="s">
-        <v>79</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -2285,7 +2440,7 @@
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="M19" s="1" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>5</v>
@@ -2296,16 +2451,16 @@
         <v>8</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -2315,7 +2470,7 @@
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>5</v>
@@ -2382,61 +2537,61 @@
         <v>3</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="H1" s="12" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="I1" s="12" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="J1" s="12" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="K1" s="12" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="L1" s="12" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="M1" s="12" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="N1" s="12" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="P1" s="12" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="S1" s="12" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="T1" s="12" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="U1" s="12" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="V1" s="12" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="W1" s="12" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="X1" s="11" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="Y1" s="11" t="s">
         <v>2</v>
@@ -2450,16 +2605,16 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>166</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="F2" s="14"/>
       <c r="G2" s="15"/>
@@ -2490,46 +2645,46 @@
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>167</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>152</v>
+        <v>113</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="H3" s="19" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="I3" s="19" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="J3" s="19" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="M3" s="19" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="N3" s="19" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="O3" s="19" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="P3" s="19"/>
       <c r="Q3" s="19"/>
@@ -2550,16 +2705,16 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>168</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E4" s="24" t="s">
-        <v>130</v>
+        <v>111</v>
       </c>
       <c r="F4" s="20"/>
       <c r="G4" s="20"/>
@@ -2604,16 +2759,16 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>169</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>128</v>
+        <v>109</v>
       </c>
       <c r="F5" s="20"/>
       <c r="G5" s="20"/>
@@ -2632,7 +2787,7 @@
       <c r="T5" s="20"/>
       <c r="U5" s="20"/>
       <c r="V5" s="20" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="W5" s="20"/>
       <c r="X5" s="20"/>
@@ -2648,16 +2803,16 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>170</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>158</v>
+        <v>119</v>
       </c>
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
@@ -2676,7 +2831,7 @@
       <c r="T6" s="20"/>
       <c r="U6" s="20"/>
       <c r="V6" s="20" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="W6" s="20"/>
       <c r="X6" s="20">
@@ -2694,16 +2849,16 @@
         <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>14</v>
+        <v>171</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>156</v>
+        <v>117</v>
       </c>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
@@ -2722,7 +2877,7 @@
       <c r="T7" s="20"/>
       <c r="U7" s="20"/>
       <c r="V7" s="20" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="W7" s="20"/>
       <c r="X7" s="20">
@@ -2740,16 +2895,16 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>172</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>157</v>
+        <v>118</v>
       </c>
       <c r="F8" s="20"/>
       <c r="G8" s="20"/>
@@ -2768,7 +2923,7 @@
       <c r="T8" s="20"/>
       <c r="U8" s="20"/>
       <c r="V8" s="20" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="W8" s="20"/>
       <c r="X8" s="20">
@@ -2786,16 +2941,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>16</v>
+        <v>173</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>159</v>
+        <v>120</v>
       </c>
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
@@ -2814,7 +2969,7 @@
       <c r="T9" s="20"/>
       <c r="U9" s="20"/>
       <c r="V9" s="20" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="W9" s="20"/>
       <c r="X9" s="20">
@@ -2832,16 +2987,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>17</v>
+        <v>174</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="F10" s="20"/>
       <c r="G10" s="20"/>
@@ -2860,7 +3015,7 @@
       <c r="T10" s="20"/>
       <c r="U10" s="20"/>
       <c r="V10" s="20" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="W10" s="20"/>
       <c r="X10" s="20">
@@ -2878,16 +3033,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
+        <v>175</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>161</v>
+        <v>122</v>
       </c>
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
@@ -2906,7 +3061,7 @@
       <c r="T11" s="20"/>
       <c r="U11" s="20"/>
       <c r="V11" s="20" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="W11" s="20"/>
       <c r="X11" s="20">
@@ -2924,16 +3079,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>176</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>162</v>
+        <v>123</v>
       </c>
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>
@@ -2952,7 +3107,7 @@
       <c r="T12" s="20"/>
       <c r="U12" s="20"/>
       <c r="V12" s="20" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="W12" s="20"/>
       <c r="X12" s="20">
@@ -2970,16 +3125,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>20</v>
+        <v>177</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>163</v>
+        <v>124</v>
       </c>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
@@ -2998,7 +3153,7 @@
       <c r="T13" s="20"/>
       <c r="U13" s="20"/>
       <c r="V13" s="20" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="W13" s="20"/>
       <c r="X13" s="20">
@@ -3016,16 +3171,16 @@
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>21</v>
+        <v>178</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>164</v>
+        <v>125</v>
       </c>
       <c r="F14" s="20"/>
       <c r="G14" s="20"/>
@@ -3044,7 +3199,7 @@
       <c r="T14" s="20"/>
       <c r="U14" s="20"/>
       <c r="V14" s="20" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="W14" s="20"/>
       <c r="X14" s="20">
@@ -3062,16 +3217,16 @@
         <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>22</v>
+        <v>179</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>165</v>
+        <v>126</v>
       </c>
       <c r="F15" s="20"/>
       <c r="G15" s="20"/>
@@ -3090,7 +3245,7 @@
       <c r="T15" s="20"/>
       <c r="U15" s="20"/>
       <c r="V15" s="20" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="W15" s="20"/>
       <c r="X15" s="20">
@@ -3108,16 +3263,16 @@
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>23</v>
+        <v>180</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>166</v>
+        <v>127</v>
       </c>
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
@@ -3136,7 +3291,7 @@
       <c r="T16" s="20"/>
       <c r="U16" s="20"/>
       <c r="V16" s="20" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="W16" s="20"/>
       <c r="X16" s="20">
@@ -3154,16 +3309,16 @@
         <v>8</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>24</v>
+        <v>181</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="F17" s="20"/>
       <c r="G17" s="20"/>
@@ -3182,7 +3337,7 @@
       <c r="T17" s="20"/>
       <c r="U17" s="20"/>
       <c r="V17" s="20" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="W17" s="20"/>
       <c r="X17" s="20">
@@ -3200,16 +3355,16 @@
         <v>8</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>80</v>
+        <v>182</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>168</v>
+        <v>129</v>
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20"/>
@@ -3228,7 +3383,7 @@
       <c r="T18" s="20"/>
       <c r="U18" s="20"/>
       <c r="V18" s="20" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="W18" s="20"/>
       <c r="X18" s="20">
@@ -3246,16 +3401,16 @@
         <v>8</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>81</v>
+        <v>183</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>169</v>
+        <v>130</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
@@ -3274,7 +3429,7 @@
       <c r="T19" s="20"/>
       <c r="U19" s="20"/>
       <c r="V19" s="20" t="s">
-        <v>154</v>
+        <v>115</v>
       </c>
       <c r="W19" s="20"/>
       <c r="X19" s="20">
@@ -3292,16 +3447,16 @@
         <v>8</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="20" t="s">
         <v>131</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="E20" s="20" t="s">
-        <v>170</v>
       </c>
       <c r="F20" s="20"/>
       <c r="G20" s="20"/>
@@ -3320,7 +3475,7 @@
       <c r="T20" s="20"/>
       <c r="U20" s="20"/>
       <c r="V20" s="20" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="W20" s="20"/>
       <c r="X20" s="20">
@@ -3338,16 +3493,16 @@
         <v>8</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E21" s="20" t="s">
         <v>132</v>
-      </c>
-      <c r="D21" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="E21" s="20" t="s">
-        <v>171</v>
       </c>
       <c r="F21" s="20"/>
       <c r="G21" s="20"/>
@@ -3366,7 +3521,7 @@
       <c r="T21" s="20"/>
       <c r="U21" s="20"/>
       <c r="V21" s="20" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="W21" s="20"/>
       <c r="X21" s="20">
@@ -3384,16 +3539,16 @@
         <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D22" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" s="20" t="s">
         <v>133</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="E22" s="20" t="s">
-        <v>172</v>
       </c>
       <c r="F22" s="20"/>
       <c r="G22" s="20"/>
@@ -3412,7 +3567,7 @@
       <c r="T22" s="20"/>
       <c r="U22" s="20"/>
       <c r="V22" s="20" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="W22" s="20"/>
       <c r="X22" s="20">
@@ -3430,16 +3585,16 @@
         <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D23" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E23" s="20" t="s">
         <v>134</v>
-      </c>
-      <c r="D23" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="E23" s="20" t="s">
-        <v>173</v>
       </c>
       <c r="F23" s="20"/>
       <c r="G23" s="20"/>
@@ -3458,7 +3613,7 @@
       <c r="T23" s="20"/>
       <c r="U23" s="20"/>
       <c r="V23" s="20" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="W23" s="20"/>
       <c r="X23" s="20">
@@ -3476,16 +3631,16 @@
         <v>8</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D24" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="E24" s="24" t="s">
         <v>135</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>101</v>
-      </c>
-      <c r="E24" s="24" t="s">
-        <v>174</v>
       </c>
       <c r="F24" s="20"/>
       <c r="G24" s="20"/>
@@ -3504,7 +3659,7 @@
       <c r="T24" s="20"/>
       <c r="U24" s="20"/>
       <c r="V24" s="20" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="W24" s="20"/>
       <c r="X24" s="20">
@@ -3522,16 +3677,16 @@
         <v>8</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E25" s="24" t="s">
         <v>136</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="E25" s="24" t="s">
-        <v>175</v>
       </c>
       <c r="F25" s="20"/>
       <c r="G25" s="20"/>
@@ -3550,7 +3705,7 @@
       <c r="T25" s="20"/>
       <c r="U25" s="20"/>
       <c r="V25" s="20" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="W25" s="22">
         <v>139000</v>
@@ -3570,16 +3725,16 @@
         <v>8</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E26" s="20" t="s">
         <v>137</v>
-      </c>
-      <c r="D26" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="E26" s="20" t="s">
-        <v>176</v>
       </c>
       <c r="F26" s="20"/>
       <c r="G26" s="20"/>
@@ -3598,7 +3753,7 @@
       <c r="T26" s="20"/>
       <c r="U26" s="20"/>
       <c r="V26" s="20" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="W26" s="22">
         <v>354000</v>
@@ -3618,16 +3773,16 @@
         <v>8</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E27" s="20" t="s">
         <v>138</v>
-      </c>
-      <c r="D27" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="E27" s="20" t="s">
-        <v>177</v>
       </c>
       <c r="F27" s="20"/>
       <c r="G27" s="20"/>
@@ -3646,7 +3801,7 @@
       <c r="T27" s="20"/>
       <c r="U27" s="20"/>
       <c r="V27" s="20" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="W27" s="22">
         <v>62350</v>
@@ -3666,16 +3821,16 @@
         <v>8</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" s="20" t="s">
         <v>139</v>
-      </c>
-      <c r="D28" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="E28" s="20" t="s">
-        <v>178</v>
       </c>
       <c r="F28" s="20"/>
       <c r="G28" s="20"/>
@@ -3694,7 +3849,7 @@
       <c r="T28" s="20"/>
       <c r="U28" s="20"/>
       <c r="V28" s="20" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="W28" s="22">
         <v>521000</v>
@@ -3714,16 +3869,16 @@
         <v>8</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="E29" s="20" t="s">
         <v>140</v>
-      </c>
-      <c r="D29" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="E29" s="20" t="s">
-        <v>179</v>
       </c>
       <c r="F29" s="20"/>
       <c r="G29" s="20"/>
@@ -3742,7 +3897,7 @@
       <c r="T29" s="20"/>
       <c r="U29" s="20"/>
       <c r="V29" s="20" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="W29" s="22">
         <v>352200</v>
@@ -3757,21 +3912,21 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:26" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>141</v>
+        <v>194</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>123</v>
+        <v>236</v>
       </c>
       <c r="F30" s="10"/>
       <c r="G30" s="19"/>
@@ -3804,16 +3959,16 @@
         <v>8</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>142</v>
+        <v>195</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E31" s="24" t="s">
-        <v>184</v>
+        <v>145</v>
       </c>
       <c r="F31" s="20"/>
       <c r="G31" s="20"/>
@@ -3832,7 +3987,7 @@
       <c r="T31" s="20"/>
       <c r="U31" s="20"/>
       <c r="V31" s="20" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="W31" s="20"/>
       <c r="X31" s="23">
@@ -3850,16 +4005,16 @@
         <v>8</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>143</v>
+        <v>196</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>183</v>
+        <v>144</v>
       </c>
       <c r="F32" s="20"/>
       <c r="G32" s="20"/>
@@ -3878,7 +4033,7 @@
       <c r="T32" s="20"/>
       <c r="U32" s="20"/>
       <c r="V32" s="20" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="W32" s="20"/>
       <c r="X32" s="23">
@@ -3896,16 +4051,16 @@
         <v>8</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>144</v>
+        <v>197</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>182</v>
+        <v>143</v>
       </c>
       <c r="F33" s="20"/>
       <c r="G33" s="20"/>
@@ -3924,7 +4079,7 @@
       <c r="T33" s="20"/>
       <c r="U33" s="20"/>
       <c r="V33" s="20" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="W33" s="20"/>
       <c r="X33" s="23">
@@ -3942,16 +4097,16 @@
         <v>8</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>145</v>
+        <v>198</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E34" s="20" t="s">
-        <v>181</v>
+        <v>142</v>
       </c>
       <c r="F34" s="20"/>
       <c r="G34" s="20"/>
@@ -3970,7 +4125,7 @@
       <c r="T34" s="20"/>
       <c r="U34" s="20"/>
       <c r="V34" s="20" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="W34" s="20"/>
       <c r="X34" s="23">
@@ -3988,16 +4143,16 @@
         <v>8</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>146</v>
+        <v>199</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E35" s="20" t="s">
-        <v>180</v>
+        <v>141</v>
       </c>
       <c r="F35" s="20"/>
       <c r="G35" s="20"/>
@@ -4016,7 +4171,7 @@
       <c r="T35" s="20"/>
       <c r="U35" s="20"/>
       <c r="V35" s="20" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="W35" s="20"/>
       <c r="X35" s="23">
@@ -4034,16 +4189,16 @@
         <v>8</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>147</v>
+        <v>200</v>
       </c>
       <c r="D36" s="20" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="F36" s="20"/>
       <c r="G36" s="20"/>
@@ -4128,61 +4283,61 @@
         <v>3</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="H1" s="26" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="I1" s="26" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="J1" s="26" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="K1" s="26" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="L1" s="26" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="M1" s="26" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="N1" s="26" t="s">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="O1" s="26" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="P1" s="26" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="Q1" s="26" t="s">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="R1" s="26" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="S1" s="26" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="T1" s="26" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="U1" s="26" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="V1" s="26" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="W1" s="26" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="X1" s="27" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="Y1" s="27" t="s">
         <v>2</v>
@@ -4196,16 +4351,16 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>9</v>
+        <v>201</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E2" s="16" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="F2" s="20"/>
       <c r="G2" s="20"/>
@@ -4236,46 +4391,46 @@
         <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>202</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>153</v>
+        <v>114</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="H3" s="19" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="I3" s="19" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
       <c r="J3" s="19" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="M3" s="19" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="N3" s="19" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="O3" s="19" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="P3" s="19"/>
       <c r="Q3" s="19"/>
@@ -4296,16 +4451,16 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>203</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="F4" s="20"/>
       <c r="G4" s="20"/>
@@ -4350,16 +4505,16 @@
         <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>204</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>155</v>
+        <v>116</v>
       </c>
       <c r="F5" s="20"/>
       <c r="G5" s="20"/>
@@ -4378,7 +4533,7 @@
       <c r="T5" s="20"/>
       <c r="U5" s="20"/>
       <c r="V5" s="20" t="s">
-        <v>104</v>
+        <v>86</v>
       </c>
       <c r="W5" s="20"/>
       <c r="X5" s="20">
@@ -4396,16 +4551,16 @@
         <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>205</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>156</v>
+        <v>117</v>
       </c>
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
@@ -4424,7 +4579,7 @@
       <c r="T6" s="20"/>
       <c r="U6" s="20"/>
       <c r="V6" s="20" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="W6" s="20"/>
       <c r="X6" s="20">
@@ -4442,16 +4597,16 @@
         <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>14</v>
+        <v>206</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E7" s="20" t="s">
-        <v>157</v>
+        <v>118</v>
       </c>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
@@ -4470,7 +4625,7 @@
       <c r="T7" s="20"/>
       <c r="U7" s="20"/>
       <c r="V7" s="20" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="W7" s="20"/>
       <c r="X7" s="20">
@@ -4488,16 +4643,16 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>207</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>159</v>
+        <v>120</v>
       </c>
       <c r="F8" s="20"/>
       <c r="G8" s="20"/>
@@ -4516,7 +4671,7 @@
       <c r="T8" s="20"/>
       <c r="U8" s="20"/>
       <c r="V8" s="20" t="s">
-        <v>105</v>
+        <v>87</v>
       </c>
       <c r="W8" s="20"/>
       <c r="X8" s="20">
@@ -4534,16 +4689,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>16</v>
+        <v>208</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E9" s="20" t="s">
-        <v>160</v>
+        <v>121</v>
       </c>
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
@@ -4562,7 +4717,7 @@
       <c r="T9" s="20"/>
       <c r="U9" s="20"/>
       <c r="V9" s="20" t="s">
-        <v>106</v>
+        <v>88</v>
       </c>
       <c r="W9" s="20"/>
       <c r="X9" s="20">
@@ -4580,16 +4735,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>17</v>
+        <v>209</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>161</v>
+        <v>122</v>
       </c>
       <c r="F10" s="20"/>
       <c r="G10" s="20"/>
@@ -4608,7 +4763,7 @@
       <c r="T10" s="20"/>
       <c r="U10" s="20"/>
       <c r="V10" s="20" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="W10" s="20"/>
       <c r="X10" s="20">
@@ -4626,16 +4781,16 @@
         <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>18</v>
+        <v>210</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>162</v>
+        <v>123</v>
       </c>
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
@@ -4654,7 +4809,7 @@
       <c r="T11" s="20"/>
       <c r="U11" s="20"/>
       <c r="V11" s="20" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="W11" s="20"/>
       <c r="X11" s="20">
@@ -4672,16 +4827,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>211</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E12" s="20" t="s">
-        <v>163</v>
+        <v>124</v>
       </c>
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>
@@ -4700,7 +4855,7 @@
       <c r="T12" s="20"/>
       <c r="U12" s="20"/>
       <c r="V12" s="20" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="W12" s="20"/>
       <c r="X12" s="20">
@@ -4718,16 +4873,16 @@
         <v>8</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>20</v>
+        <v>212</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E13" s="20" t="s">
-        <v>164</v>
+        <v>125</v>
       </c>
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
@@ -4746,7 +4901,7 @@
       <c r="T13" s="20"/>
       <c r="U13" s="20"/>
       <c r="V13" s="20" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="W13" s="20"/>
       <c r="X13" s="20">
@@ -4764,16 +4919,16 @@
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>21</v>
+        <v>213</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E14" s="20" t="s">
-        <v>165</v>
+        <v>126</v>
       </c>
       <c r="F14" s="20"/>
       <c r="G14" s="20"/>
@@ -4792,7 +4947,7 @@
       <c r="T14" s="20"/>
       <c r="U14" s="20"/>
       <c r="V14" s="20" t="s">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="W14" s="20"/>
       <c r="X14" s="20">
@@ -4810,16 +4965,16 @@
         <v>8</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>22</v>
+        <v>214</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>166</v>
+        <v>127</v>
       </c>
       <c r="F15" s="20"/>
       <c r="G15" s="20"/>
@@ -4838,7 +4993,7 @@
       <c r="T15" s="20"/>
       <c r="U15" s="20"/>
       <c r="V15" s="20" t="s">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="W15" s="20"/>
       <c r="X15" s="20">
@@ -4856,16 +5011,16 @@
         <v>8</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>23</v>
+        <v>215</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
@@ -4884,7 +5039,7 @@
       <c r="T16" s="20"/>
       <c r="U16" s="20"/>
       <c r="V16" s="20" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="W16" s="20"/>
       <c r="X16" s="20">
@@ -4902,16 +5057,16 @@
         <v>8</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>24</v>
+        <v>216</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E17" s="24" t="s">
-        <v>168</v>
+        <v>129</v>
       </c>
       <c r="F17" s="20"/>
       <c r="G17" s="20"/>
@@ -4930,7 +5085,7 @@
       <c r="T17" s="20"/>
       <c r="U17" s="20"/>
       <c r="V17" s="20" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="W17" s="20"/>
       <c r="X17" s="20">
@@ -4948,16 +5103,16 @@
         <v>8</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>80</v>
+        <v>217</v>
       </c>
       <c r="D18" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>169</v>
+        <v>130</v>
       </c>
       <c r="F18" s="20"/>
       <c r="G18" s="20"/>
@@ -4976,7 +5131,7 @@
       <c r="T18" s="20"/>
       <c r="U18" s="20"/>
       <c r="V18" s="20" t="s">
-        <v>154</v>
+        <v>115</v>
       </c>
       <c r="W18" s="20"/>
       <c r="X18" s="20">
@@ -4994,16 +5149,16 @@
         <v>8</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>81</v>
+        <v>218</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E19" s="20" t="s">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
@@ -5022,7 +5177,7 @@
       <c r="T19" s="20"/>
       <c r="U19" s="20"/>
       <c r="V19" s="20" t="s">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="W19" s="20"/>
       <c r="X19" s="20">
@@ -5040,16 +5195,16 @@
         <v>8</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>131</v>
+        <v>219</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>171</v>
+        <v>132</v>
       </c>
       <c r="F20" s="20"/>
       <c r="G20" s="20"/>
@@ -5068,7 +5223,7 @@
       <c r="T20" s="20"/>
       <c r="U20" s="20"/>
       <c r="V20" s="20" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="W20" s="20"/>
       <c r="X20" s="20">
@@ -5086,16 +5241,16 @@
         <v>8</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>132</v>
+        <v>220</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E21" s="20" t="s">
-        <v>172</v>
+        <v>133</v>
       </c>
       <c r="F21" s="20"/>
       <c r="G21" s="20"/>
@@ -5114,7 +5269,7 @@
       <c r="T21" s="20"/>
       <c r="U21" s="20"/>
       <c r="V21" s="20" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="W21" s="20"/>
       <c r="X21" s="20">
@@ -5132,16 +5287,16 @@
         <v>8</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>133</v>
+        <v>221</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E22" s="20" t="s">
-        <v>173</v>
+        <v>134</v>
       </c>
       <c r="F22" s="20"/>
       <c r="G22" s="20"/>
@@ -5160,7 +5315,7 @@
       <c r="T22" s="20"/>
       <c r="U22" s="20"/>
       <c r="V22" s="20" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="W22" s="20"/>
       <c r="X22" s="20">
@@ -5178,16 +5333,16 @@
         <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>134</v>
+        <v>222</v>
       </c>
       <c r="D23" s="20" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>174</v>
+        <v>135</v>
       </c>
       <c r="F23" s="20"/>
       <c r="G23" s="20"/>
@@ -5206,7 +5361,7 @@
       <c r="T23" s="20"/>
       <c r="U23" s="20"/>
       <c r="V23" s="20" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="W23" s="20"/>
       <c r="X23" s="20">
@@ -5224,16 +5379,16 @@
         <v>8</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>135</v>
+        <v>223</v>
       </c>
       <c r="D24" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>175</v>
+        <v>136</v>
       </c>
       <c r="F24" s="20"/>
       <c r="G24" s="20"/>
@@ -5252,7 +5407,7 @@
       <c r="T24" s="20"/>
       <c r="U24" s="20"/>
       <c r="V24" s="20" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="W24" s="22">
         <v>580000</v>
@@ -5272,16 +5427,16 @@
         <v>8</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>136</v>
+        <v>224</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>176</v>
+        <v>137</v>
       </c>
       <c r="F25" s="20"/>
       <c r="G25" s="20"/>
@@ -5300,7 +5455,7 @@
       <c r="T25" s="20"/>
       <c r="U25" s="20"/>
       <c r="V25" s="20" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="W25" s="22">
         <v>354000</v>
@@ -5311,23 +5466,25 @@
       <c r="Y25" s="20" t="b">
         <v>1</v>
       </c>
-      <c r="Z25" s="1"/>
+      <c r="Z25" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="26" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>137</v>
+        <v>225</v>
       </c>
       <c r="D26" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="F26" s="20"/>
       <c r="G26" s="20"/>
@@ -5346,7 +5503,7 @@
       <c r="T26" s="20"/>
       <c r="U26" s="20"/>
       <c r="V26" s="20" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="W26" s="22">
         <v>62350</v>
@@ -5366,16 +5523,16 @@
         <v>8</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>138</v>
+        <v>226</v>
       </c>
       <c r="D27" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E27" s="20" t="s">
-        <v>178</v>
+        <v>139</v>
       </c>
       <c r="F27" s="20"/>
       <c r="G27" s="20"/>
@@ -5394,7 +5551,7 @@
       <c r="T27" s="20"/>
       <c r="U27" s="20"/>
       <c r="V27" s="20" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="W27" s="22">
         <v>1700000</v>
@@ -5414,16 +5571,16 @@
         <v>8</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>139</v>
+        <v>227</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>179</v>
+        <v>140</v>
       </c>
       <c r="F28" s="20"/>
       <c r="G28" s="20"/>
@@ -5442,7 +5599,7 @@
       <c r="T28" s="20"/>
       <c r="U28" s="20"/>
       <c r="V28" s="20" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="W28" s="22">
         <v>822000</v>
@@ -5457,21 +5614,21 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:26" ht="29" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>141</v>
+        <v>228</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>123</v>
+        <v>236</v>
       </c>
       <c r="F29" s="20"/>
       <c r="G29" s="20"/>
@@ -5504,16 +5661,16 @@
         <v>8</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>142</v>
+        <v>229</v>
       </c>
       <c r="D30" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E30" s="24" t="s">
-        <v>184</v>
+        <v>145</v>
       </c>
       <c r="F30" s="20"/>
       <c r="G30" s="20"/>
@@ -5532,7 +5689,7 @@
       <c r="T30" s="20"/>
       <c r="U30" s="20"/>
       <c r="V30" s="20" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="W30" s="22">
         <v>580000</v>
@@ -5552,16 +5709,16 @@
         <v>8</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>143</v>
+        <v>230</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>183</v>
+        <v>144</v>
       </c>
       <c r="F31" s="20"/>
       <c r="G31" s="20"/>
@@ -5580,7 +5737,7 @@
       <c r="T31" s="20"/>
       <c r="U31" s="20"/>
       <c r="V31" s="20" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="W31" s="22">
         <v>354000</v>
@@ -5600,16 +5757,16 @@
         <v>8</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>144</v>
+        <v>231</v>
       </c>
       <c r="D32" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E32" s="20" t="s">
-        <v>182</v>
+        <v>143</v>
       </c>
       <c r="F32" s="20"/>
       <c r="G32" s="20"/>
@@ -5628,7 +5785,7 @@
       <c r="T32" s="20"/>
       <c r="U32" s="20"/>
       <c r="V32" s="20" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="W32" s="22">
         <v>62350</v>
@@ -5648,16 +5805,16 @@
         <v>8</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>145</v>
+        <v>232</v>
       </c>
       <c r="D33" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E33" s="20" t="s">
-        <v>181</v>
+        <v>142</v>
       </c>
       <c r="F33" s="20"/>
       <c r="G33" s="20"/>
@@ -5676,7 +5833,7 @@
       <c r="T33" s="20"/>
       <c r="U33" s="20"/>
       <c r="V33" s="20" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="W33" s="22">
         <v>1700000</v>
@@ -5696,16 +5853,16 @@
         <v>8</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>146</v>
+        <v>233</v>
       </c>
       <c r="D34" s="20" t="s">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="E34" s="20" t="s">
-        <v>180</v>
+        <v>141</v>
       </c>
       <c r="F34" s="20"/>
       <c r="G34" s="20"/>
@@ -5724,7 +5881,7 @@
       <c r="T34" s="20"/>
       <c r="U34" s="20"/>
       <c r="V34" s="20" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="W34" s="22">
         <v>822000</v>
@@ -5744,16 +5901,16 @@
         <v>8</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>147</v>
+        <v>234</v>
       </c>
       <c r="D35" s="20" t="s">
-        <v>129</v>
+        <v>110</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>127</v>
+        <v>108</v>
       </c>
       <c r="F35" s="20"/>
       <c r="G35" s="20"/>
@@ -5782,6 +5939,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cost Calculator Module resolved failed testcases
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/16_Cost_Calculator/CostCalculator/01_CostCalculatorTest.xlsx
+++ b/src/test/resources/testdata/Modules/16_Cost_Calculator/CostCalculator/01_CostCalculatorTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\16_Cost_Calculator\CostCalculator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C8BC92-E8B7-4CA3-A8EE-0C6AE4FC0452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71BE81E2-E1AB-4FB1-A7F9-CEF005BAE825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="201">
   <si>
     <t>TESTCASE_ID</t>
   </si>
@@ -694,6 +694,13 @@
 click_back
 click_exit_ok
 navigatebacktodashboardpage</t>
+  </si>
+  <si>
+    <t>clickon_add_dreamgiftbtn
+dreamgift_get_dreamgiftname
+dreamgift_open_dreamgift
+dreamgift_open_dreamgift
+verify_selecteddreamgift_name</t>
   </si>
 </sst>
 </file>
@@ -2547,7 +2554,7 @@
         <v>75</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>118</v>
+        <v>200</v>
       </c>
       <c r="F27" s="11"/>
       <c r="G27" s="11"/>

</xml_diff>